<commit_message>
Modification acompte avec ajout des factures.
</commit_message>
<xml_diff>
--- a/Documents/Acomptes/Acomptes_2405.xlsx
+++ b/Documents/Acomptes/Acomptes_2405.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Acomptes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F949B10D-1CB3-4625-AE63-DAB96A531BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F9F9DB6-12DE-4C5A-A079-996DEC54B3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2325" yWindow="2235" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{7AA76E0D-F087-4492-9963-C5C0844E84C2}"/>
+    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{322EFC9B-DAF8-4336-9062-7DEE3A79D121}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
     <sheet name="SCAF GRANGE DE VAIVRE    " sheetId="2" r:id="rId2"/>
     <sheet name="SCAF BRESSE JURASSIENNE  " sheetId="3" r:id="rId3"/>
-    <sheet name="COOP MONTS DE JOUX" sheetId="4" r:id="rId4"/>
+    <sheet name="ANDELOT" sheetId="4" r:id="rId4"/>
     <sheet name="SCAF LONGEVELLE-RUSSEY   " sheetId="5" r:id="rId5"/>
-    <sheet name="COOP MONTS DE JOUX       " sheetId="6" r:id="rId6"/>
+    <sheet name="GD COMBE CHATELEU        " sheetId="6" r:id="rId6"/>
     <sheet name="SCAF LAVANS VUILLAFANS   " sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -42,12 +42,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="54">
-  <si>
-    <t xml:space="preserve">M PONCET FREDERIC        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF GRANGE DE VAIVRE    </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="45">
+  <si>
+    <t>Mr Frédéric PONCET</t>
   </si>
   <si>
     <t xml:space="preserve">                         </t>
@@ -110,25 +107,22 @@
     <t>Service Comptabilité</t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39029 50546581010 50</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39029 50546581010 11</t>
   </si>
   <si>
     <t>CAFC SALINS LES BAINS   , la somme de</t>
   </si>
   <si>
-    <t xml:space="preserve">M BUATOIS ANTHONY        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF BRESSE JURASSIENNE  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 PLACE DE LA MAIRIE     </t>
+    <t>Mr Benoit COTE</t>
+  </si>
+  <si>
+    <t>3 Pace de la Mairie</t>
   </si>
   <si>
     <t xml:space="preserve">39140  DESNES                  </t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39023 40357496000 40</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 12506 39023 40357496000 54</t>
   </si>
   <si>
     <t>CAFC POLIGNY            , la somme de</t>
@@ -137,34 +131,28 @@
     <t>ATELIER ANDELOT</t>
   </si>
   <si>
-    <t>COOP MONTS DE JOUX</t>
-  </si>
-  <si>
-    <t>36, Rue Laurent TROUTET</t>
-  </si>
-  <si>
-    <t>25560 BANNANS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PS : Nous virons ce jour, sur votre compte N° 0 0  </t>
-  </si>
-  <si>
-    <t>, la somme de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mr DEVAUX JOHANN         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF LONGEVELLE/RUSSEY   </t>
+    <t>36 Rue Laurent Troutet</t>
+  </si>
+  <si>
+    <t>25560  BANANS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PS : Nous virons ce jour, sur votre compte N° 0 0               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">                        , la somme de</t>
+  </si>
+  <si>
+    <t>Mr Johann DEVAUX</t>
   </si>
   <si>
     <t xml:space="preserve">2, rue du Conot          </t>
   </si>
   <si>
-    <t>25380 CHARMOILLE</t>
-  </si>
-  <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 12506 20017 11707951010 11</t>
+    <t xml:space="preserve">25380  CHARMOILLE              </t>
+  </si>
+  <si>
+    <t>PS : Nous virons ce jour, sur votre compte N° 12506 20017 11707951010 37</t>
   </si>
   <si>
     <t>CAFC SANCEY LE GRAND    , la somme de</t>
@@ -173,34 +161,19 @@
     <t>Atelier Gd Combe Chateleu</t>
   </si>
   <si>
-    <t xml:space="preserve">COOP MONTS DE JOUX       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">36 Rue Laurent TROUTET   </t>
-  </si>
-  <si>
     <t xml:space="preserve">25560 BANNANS                  </t>
   </si>
   <si>
-    <t xml:space="preserve">PS : Nous virons ce jour, sur votre compte N° 0 0               </t>
-  </si>
-  <si>
-    <t xml:space="preserve">                        , la somme de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MR JOANY LEPINE          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCAF LAVANS VUILLAFANS   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6, Chemin des Clos Ronds </t>
+    <t>Mr Joany LEPINE</t>
+  </si>
+  <si>
+    <t>6 Chemin des Clos Ronds</t>
   </si>
   <si>
     <t xml:space="preserve">25380  LAVANS VUILLAFANS       </t>
   </si>
   <si>
-    <t>PS : Nous virons ce jour, sur votre compte N° 10807 6 22321737995 22</t>
+    <t>PS : Nous virons ce jour, sur votre compte N° 10807 6 22321737995 58</t>
   </si>
   <si>
     <t>BNP ORNANS              , la somme de</t>
@@ -629,7 +602,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96DB6243-0E78-4646-9E4C-DF8F8DA178DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF3347E5-90E4-4A47-BF29-C6A288C161B0}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -638,8 +611,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2801D124-3733-4DA5-8229-2509AC9D39ED}">
-  <dimension ref="A10:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB980317-DF85-4D91-A67A-AEB299B4B965}">
+  <dimension ref="A11:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -655,70 +628,65 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4">
         <v>104</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5">
         <v>3.6669999999999998</v>
       </c>
       <c r="F28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -728,7 +696,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -737,13 +705,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -753,7 +721,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -762,32 +730,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -800,8 +768,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C57D3C8D-F8C9-4F6A-98DB-8A59F8978868}">
-  <dimension ref="A10:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{601C240D-19D8-4573-A2B3-A0AB9C07E006}">
+  <dimension ref="A11:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -817,70 +785,65 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4">
         <v>392</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5">
         <v>14.491</v>
       </c>
       <c r="F28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -890,7 +853,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -899,13 +862,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -915,7 +878,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -924,32 +887,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -962,8 +925,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCB93CDF-2345-4EF2-B4AC-F970ADC0708C}">
-  <dimension ref="A10:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D0B43F2-23F7-43BE-AE43-ED42EBB98ED8}">
+  <dimension ref="A11:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -979,70 +942,65 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4">
         <v>288</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5">
         <v>11.634</v>
       </c>
       <c r="F28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1052,7 +1010,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1061,13 +1019,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1077,7 +1035,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1086,32 +1044,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1124,8 +1082,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8FEC72F-B3C2-4C65-B65B-B5571E9B54F0}">
-  <dimension ref="A10:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BE94C46-993D-4A1E-8B24-B7D21801BADA}">
+  <dimension ref="A11:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -1141,70 +1099,65 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4">
         <v>672</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5">
         <v>25.975999999999999</v>
       </c>
       <c r="F28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1214,7 +1167,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1223,13 +1176,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1239,7 +1192,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1248,32 +1201,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1286,8 +1239,8 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{444E4C0A-EB57-44D1-83EA-AF4567D1F929}">
-  <dimension ref="A10:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC97B1F5-4391-43E8-BC58-F8ED34F16275}">
+  <dimension ref="A11:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -1303,70 +1256,65 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4">
         <v>312</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5">
         <v>12.250999999999999</v>
       </c>
       <c r="F28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1376,7 +1324,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1385,13 +1333,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1401,7 +1349,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1410,32 +1358,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1448,8 +1396,8 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD3F257-6579-4103-A20C-50770285AE09}">
-  <dimension ref="A10:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EF68691-3B7A-43ED-8FF3-6A5F89DC4313}">
+  <dimension ref="A11:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -1465,70 +1413,65 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F10" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4">
         <v>531</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E28" s="5">
         <v>21.297000000000001</v>
       </c>
       <c r="F28" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>10</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1538,7 +1481,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1547,13 +1490,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="I31" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1563,7 +1506,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1572,32 +1515,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>

</xml_diff>

<commit_message>
Arrondi à deux chiffres pour la prime dans le calcul du montant et ajout des coop dans les select pour les acomptes et les classements
</commit_message>
<xml_diff>
--- a/Documents/Acomptes/Acomptes_2405.xlsx
+++ b/Documents/Acomptes/Acomptes_2405.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Acomptes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F9F9DB6-12DE-4C5A-A079-996DEC54B3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B58B837C-7A6B-45EC-9215-CD93A542B865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{322EFC9B-DAF8-4336-9062-7DEE3A79D121}"/>
+    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{911293AD-42CC-4B40-AA3D-53F6B9A3215B}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="50">
+  <si>
+    <t>SCAF DE LA FRUITIERE DU VAL DE LOUE</t>
+  </si>
   <si>
     <t>Mr Frédéric PONCET</t>
   </si>
@@ -113,6 +116,9 @@
     <t>CAFC SALINS LES BAINS   , la somme de</t>
   </si>
   <si>
+    <t>SCAF BRESSE JURASSIENNE</t>
+  </si>
+  <si>
     <t>Mr Benoit COTE</t>
   </si>
   <si>
@@ -128,6 +134,9 @@
     <t>CAFC POLIGNY            , la somme de</t>
   </si>
   <si>
+    <t>COOPERATIVE DES MONTS DE JOUX</t>
+  </si>
+  <si>
     <t>ATELIER ANDELOT</t>
   </si>
   <si>
@@ -143,6 +152,9 @@
     <t xml:space="preserve">                        , la somme de</t>
   </si>
   <si>
+    <t>SCAF DE LONGEVELLE</t>
+  </si>
+  <si>
     <t>Mr Johann DEVAUX</t>
   </si>
   <si>
@@ -162,6 +174,9 @@
   </si>
   <si>
     <t xml:space="preserve">25560 BANNANS                  </t>
+  </si>
+  <si>
+    <t>SCAF DE LAVANS VUILLAFANS</t>
   </si>
   <si>
     <t>Mr Joany LEPINE</t>
@@ -602,7 +617,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF3347E5-90E4-4A47-BF29-C6A288C161B0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F343C966-6B4A-46AE-A8DB-AE4C0899C4B9}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -611,8 +626,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB980317-DF85-4D91-A67A-AEB299B4B965}">
-  <dimension ref="A11:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCB0BF9E-6ABE-4FDD-89DA-1733FE16F304}">
+  <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -628,65 +643,70 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>104</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>3.6669999999999998</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -696,7 +716,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -705,13 +725,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -721,7 +741,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -730,32 +750,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -768,8 +788,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{601C240D-19D8-4573-A2B3-A0AB9C07E006}">
-  <dimension ref="A11:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94174584-9FBB-4C75-B54B-2D613EACFE91}">
+  <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -785,65 +805,70 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>392</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>14.491</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -853,7 +878,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -862,13 +887,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -878,7 +903,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -887,32 +912,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -925,8 +950,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D0B43F2-23F7-43BE-AE43-ED42EBB98ED8}">
-  <dimension ref="A11:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C55F4DD-F919-4B85-A6CF-4E4FA2DFC2CC}">
+  <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -942,65 +967,70 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>288</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>11.634</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1010,7 +1040,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1019,13 +1049,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1035,7 +1065,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1044,32 +1074,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1082,8 +1112,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BE94C46-993D-4A1E-8B24-B7D21801BADA}">
-  <dimension ref="A11:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8FE4A7A-BD75-4245-9C61-43D08BBAD45A}">
+  <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -1099,65 +1129,70 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>672</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>25.975999999999999</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1167,7 +1202,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1176,13 +1211,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1192,7 +1227,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1201,32 +1236,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1239,8 +1274,8 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC97B1F5-4391-43E8-BC58-F8ED34F16275}">
-  <dimension ref="A11:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9FB4597-BD17-4209-A821-65B41C2CC73E}">
+  <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -1256,65 +1291,70 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>312</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>12.250999999999999</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1324,7 +1364,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1333,13 +1373,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1349,7 +1389,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1358,32 +1398,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1396,8 +1436,8 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EF68691-3B7A-43ED-8FF3-6A5F89DC4313}">
-  <dimension ref="A11:J47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF924947-FC59-4FAD-A827-5DFEE78BE71A}">
+  <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
@@ -1413,65 +1453,70 @@
     <col min="11" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
+    <row r="10" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F10" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C28" s="4">
         <v>531</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E28" s="5">
         <v>21.297000000000001</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1481,7 +1526,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1490,13 +1535,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1506,7 +1551,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1515,32 +1560,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>

</xml_diff>

<commit_message>
Modification des tailles des colonnes Excel.
</commit_message>
<xml_diff>
--- a/Documents/Acomptes/Acomptes_2405.xlsx
+++ b/Documents/Acomptes/Acomptes_2405.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Acomptes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B58B837C-7A6B-45EC-9215-CD93A542B865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{90764CD6-8A7C-410F-9CEB-0F14D5E18785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{911293AD-42CC-4B40-AA3D-53F6B9A3215B}"/>
+    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{8B1FA1D9-F533-4E9F-9BFE-C4480C24B600}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -617,7 +617,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F343C966-6B4A-46AE-A8DB-AE4C0899C4B9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F0A8B1-C680-4FAF-92ED-D01BD28C7E0E}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -626,11 +626,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCB0BF9E-6ABE-4FDD-89DA-1733FE16F304}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4C8A94-E726-4829-9FAB-1363360B688E}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
@@ -788,11 +788,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94174584-9FBB-4C75-B54B-2D613EACFE91}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85CFA2A0-D0ED-4111-8C79-DFF3C487CC20}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
@@ -950,11 +950,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C55F4DD-F919-4B85-A6CF-4E4FA2DFC2CC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79BF07A-1916-48DC-9645-C488BB81FDC9}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
@@ -1112,11 +1112,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8FE4A7A-BD75-4245-9C61-43D08BBAD45A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{859FA6F4-5D86-40D1-BB12-B561C86E3981}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
@@ -1274,11 +1274,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9FB4597-BD17-4209-A821-65B41C2CC73E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58402EDC-A299-47DA-ADA3-1C5DC645A2E4}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>
@@ -1436,11 +1436,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF924947-FC59-4FAD-A827-5DFEE78BE71A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2B7556-607E-4D29-BA25-50A8B0509416}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="4.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.42578125" style="1" customWidth="1"/>

</xml_diff>

<commit_message>
Ouverture des fichiers après la sauvegarde.
</commit_message>
<xml_diff>
--- a/Documents/Acomptes/Acomptes_2405.xlsx
+++ b/Documents/Acomptes/Acomptes_2405.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Acomptes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{90764CD6-8A7C-410F-9CEB-0F14D5E18785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D90F2D5-B6EA-488F-9FA6-C42450F28329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24390" yWindow="2685" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{8B1FA1D9-F533-4E9F-9BFE-C4480C24B600}"/>
+    <workbookView xWindow="-24225" yWindow="3315" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{5B71382D-5A4B-41A0-B450-39DC37D40260}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -617,7 +617,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F0A8B1-C680-4FAF-92ED-D01BD28C7E0E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE588C4-09A2-4A67-9807-20E3F0B69954}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -626,7 +626,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4C8A94-E726-4829-9FAB-1363360B688E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7894E0BE-020B-424B-AA6E-24D3168BD143}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -788,7 +788,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85CFA2A0-D0ED-4111-8C79-DFF3C487CC20}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074C6C21-D034-4C1A-B4B0-877F2446B08E}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -950,7 +950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A79BF07A-1916-48DC-9645-C488BB81FDC9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51546540-5B55-44B3-95E2-A65308B4503F}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1112,7 +1112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{859FA6F4-5D86-40D1-BB12-B561C86E3981}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA3FF2D6-F455-401B-BD99-12EEE70CD344}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1274,7 +1274,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58402EDC-A299-47DA-ADA3-1C5DC645A2E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6939138-5703-47AB-85DA-9A901425BBDC}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1436,7 +1436,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2B7556-607E-4D29-BA25-50A8B0509416}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF271F0-72A4-4656-B833-AC3EABB0F7E1}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Modification d'après les instructions de Patricia.
</commit_message>
<xml_diff>
--- a/Documents/Acomptes/Acomptes_2405.xlsx
+++ b/Documents/Acomptes/Acomptes_2405.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dossier Dev\Informatique\Gestcom\Documents\Acomptes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3D90F2D5-B6EA-488F-9FA6-C42450F28329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{142A6E75-C208-4D68-A77C-CBD18A069C40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24225" yWindow="3315" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{5B71382D-5A4B-41A0-B450-39DC37D40260}"/>
+    <workbookView xWindow="3765" yWindow="2370" windowWidth="21600" windowHeight="11295" firstSheet="4" activeTab="6" xr2:uid="{2EA45457-51CA-4055-93DE-DC82EBFFE905}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="52">
   <si>
     <t>SCAF DE LA FRUITIERE DU VAL DE LOUE</t>
   </si>
@@ -56,6 +56,9 @@
     <t xml:space="preserve">39600 GRANGE DE VAIVRE         </t>
   </si>
   <si>
+    <t>Le 20 Juillet 2024</t>
+  </si>
+  <si>
     <t xml:space="preserve">      TB/PB</t>
   </si>
   <si>
@@ -65,7 +68,19 @@
     <t xml:space="preserve">          Nous vous prions de bien vouloir trouver ci-dessous, le détail</t>
   </si>
   <si>
-    <t>du premier acompte sur votre lot de fabrication MAI 2024</t>
+    <r>
+      <t xml:space="preserve">du premier acompte sur votre lot de fabrication </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>MAI 2024</t>
+    </r>
   </si>
   <si>
     <t>-</t>
@@ -162,6 +177,9 @@
   </si>
   <si>
     <t xml:space="preserve">25380  CHARMOILLE              </t>
+  </si>
+  <si>
+    <t>Le 08 Juillet 2024</t>
   </si>
   <si>
     <t>PS : Nous virons ce jour, sur votre compte N° 12506 20017 11707951010 37</t>
@@ -617,7 +635,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE588C4-09A2-4A67-9807-20E3F0B69954}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B52AFA37-00FD-4D22-92F9-14154F10557B}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -626,7 +644,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7894E0BE-020B-424B-AA6E-24D3168BD143}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ECA547AB-5455-4131-BC9E-516FDF610B8B}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -665,48 +683,51 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4">
         <v>104</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5">
         <v>3.6669999999999998</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -716,7 +737,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -725,13 +746,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -741,7 +762,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -750,32 +771,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -788,7 +809,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074C6C21-D034-4C1A-B4B0-877F2446B08E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{181CB143-91C9-4C64-AE40-EF2915EB374C}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -807,68 +828,71 @@
   <sheetData>
     <row r="10" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4">
         <v>392</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5">
         <v>14.491</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -878,7 +902,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -887,13 +911,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -903,7 +927,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -912,32 +936,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -950,7 +974,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51546540-5B55-44B3-95E2-A65308B4503F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61643867-811F-46CD-8F99-6FA335FC8726}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -969,68 +993,71 @@
   <sheetData>
     <row r="10" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4">
         <v>288</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5">
         <v>11.634</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1040,7 +1067,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1049,13 +1076,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1065,7 +1092,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1074,32 +1101,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1112,7 +1139,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA3FF2D6-F455-401B-BD99-12EEE70CD344}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3C80093-5463-4972-B749-8A8AADF34B62}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1131,68 +1158,71 @@
   <sheetData>
     <row r="10" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4">
         <v>672</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5">
         <v>25.975999999999999</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1202,7 +1232,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1211,13 +1241,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1227,7 +1257,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1236,32 +1266,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1274,7 +1304,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6939138-5703-47AB-85DA-9A901425BBDC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20EBCF03-1304-4A98-A0FA-F74A28D1040E}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1293,68 +1323,71 @@
   <sheetData>
     <row r="10" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4">
         <v>312</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5">
         <v>12.250999999999999</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1364,7 +1397,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1373,13 +1406,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1389,7 +1422,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1398,32 +1431,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>
@@ -1436,7 +1469,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AF271F0-72A4-4656-B833-AC3EABB0F7E1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F134D99E-D057-4CE9-B05C-2602BE289975}">
   <dimension ref="A10:J47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1455,68 +1488,71 @@
   <sheetData>
     <row r="10" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F10" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F11" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="6:6" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B28" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4">
         <v>531</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5">
         <v>21.297000000000001</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H28" s="8">
         <v>6750</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J28" s="11">
         <f>ROUND(+E28*H28, 2)</f>
@@ -1526,7 +1562,7 @@
     <row r="29" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F30" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" s="8">
         <f>+J28</f>
@@ -1535,13 +1571,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F31" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J31" s="12">
         <f>ROUND(+J30*H31/100, 2)</f>
@@ -1551,7 +1587,7 @@
     <row r="32" spans="1:10" ht="4.1500000000000004" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="F33" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J33" s="13">
         <f>SUM(J30:J31)</f>
@@ -1560,32 +1596,32 @@
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B37" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B38" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="H40" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B46" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J47" s="10">
         <f>+J33</f>

</xml_diff>